<commit_message>
feat: anonymize internal CLIDs with open-source IDs (CL00100-CL00146)
</commit_message>
<xml_diff>
--- a/examples/LargeDrugCombo_Goetz_Cancers_2024/raw_data/Project41.Belva.S01.manifest.xlsx
+++ b/examples/LargeDrugCombo_Goetz_Cancers_2024/raw_data/Project41.Belva.S01.manifest.xlsx
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CL587227</t>
+          <t>CL00119</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -461,7 +461,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CL586309</t>
+          <t>CL00130</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -481,7 +481,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CL586144</t>
+          <t>CL00142</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -501,7 +501,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CL584727</t>
+          <t>CL00108</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -521,7 +521,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CL131257</t>
+          <t>CL00106</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -541,7 +541,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CL586028</t>
+          <t>CL00131</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -561,7 +561,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CL586613</t>
+          <t>CL00116</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -581,7 +581,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CL587686</t>
+          <t>CL00111</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -601,7 +601,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CL131311</t>
+          <t>CL00105</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -621,7 +621,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CL131382</t>
+          <t>CL00124</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -641,7 +641,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CL131336</t>
+          <t>CL00118</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -661,7 +661,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CL586618</t>
+          <t>CL00120</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -681,7 +681,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CL131107</t>
+          <t>CL00138</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -701,7 +701,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CL583906</t>
+          <t>CL00109</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -721,7 +721,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CL586020</t>
+          <t>CL00136</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -741,7 +741,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CL586029</t>
+          <t>CL00140</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -761,7 +761,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CL586086</t>
+          <t>CL00135</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -781,7 +781,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CL586568</t>
+          <t>CL00127</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -801,7 +801,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CL586292</t>
+          <t>CL00145</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -821,7 +821,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CL131111</t>
+          <t>CL00129</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -841,7 +841,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CL586813</t>
+          <t>CL00117</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -861,7 +861,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CL131109</t>
+          <t>CL00125</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -881,7 +881,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CL585679</t>
+          <t>CL00104</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CL586959</t>
+          <t>CL00122</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -921,7 +921,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CL586650</t>
+          <t>CL00134</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -941,7 +941,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CL586090</t>
+          <t>CL00144</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -961,7 +961,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CL586143</t>
+          <t>CL00110</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -981,7 +981,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CL587462</t>
+          <t>CL00107</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1001,7 +1001,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CL586497</t>
+          <t>CL00146</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1021,7 +1021,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CL586612</t>
+          <t>CL00115</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1041,7 +1041,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CL131317</t>
+          <t>CL00133</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1061,7 +1061,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CL586596</t>
+          <t>CL00128</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1081,7 +1081,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CL586098</t>
+          <t>CL00137</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1101,7 +1101,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CL587106</t>
+          <t>CL00143</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1121,7 +1121,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CL586080</t>
+          <t>CL00126</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1141,7 +1141,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CL586647</t>
+          <t>CL00139</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1161,7 +1161,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CL587482</t>
+          <t>CL00123</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1181,7 +1181,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CL131105</t>
+          <t>CL00113</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1201,7 +1201,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CL586084</t>
+          <t>CL00112</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1221,7 +1221,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CL586108</t>
+          <t>CL00114</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CL587138</t>
+          <t>CL00141</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1261,7 +1261,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CL586619</t>
+          <t>CL00132</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1281,7 +1281,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CL586965</t>
+          <t>CL00121</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">

</xml_diff>